<commit_message>
Session 11: Vercel deploy, generate.py JSON robustness + B-10/B-11 kind enforcement, scale test batch
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -2542,6 +2542,114 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B59" s="19" t="inlineStr">
+        <is>
+          <t>Vercel deployment — next.config.ts + GitHub init</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Added outputFileTracingIncludes to web/next.config.ts so Vercel bundles data/events/**/* in the serverless function. Initialised git repo, pushed to GitHub (Ephemiral/Newsroom). Deployed to Vercel; permanent public URL available for external validators.</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>localtunnel was unreliable; reviewers needed a stable URL that works without keeping a laptop running</t>
+        </is>
+      </c>
+      <c r="E59" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude (Cowork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>Generate — JSON parse robustness fix</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>Rewrote _parse_response() in pipeline/generate/generate.py to match extract.py: strips markdown fences, repairs truncated output (stop_reason==max_tokens), falls back to json_repair library. Previously used bare json.loads() which crashed on minor model output malformation.</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>First scale test run failed with JSONDecodeError on evt_014 generate stage</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>Claude (Cowork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>Scale test — 3 new events processed</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Ran evt_2026_06_04_014 (Israel Day Parade/Smotrich, 17 art), evt_2026_06_04_062 (US-Iran ceasefire, 23 art), evt_2026_06_04_066 (Iranian drone/Kuwait, 12 art) through full pipeline. Total events: 9. All viewable at newsroom-sand-seven.vercel.app.</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>M9 scale target is 20-30 events; now at 9</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude (Cowork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>B-10/B-11 — Generate stage kind enforcement</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>Two bugs identified and fixed in pipeline/generate/generate.py: (1) B-10: model was returning claim_ids:[] in all paragraph supports, breaking downstream validation. (2) B-11: model labelled paragraphs kind=contested based on topic dispute rather than outlet-level disagreement. Fix: added ⚠ CONTESTED_BY STATUS header in _build_claims_block() when no claims have contested_by populated; added _enforce_paragraph_kinds() post-generation guard that reclassifies contested→framing when no cited claim has contested_by non-empty (or claim_ids is empty). Logged as B-10/B-11 in Master Doc §13.</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>evt_062 had 0 outlet-level disputes yet 4 contested paragraphs — readers were misled</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude (Cowork)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Session 13: B-12 clustering backlog flagged; 1 new event; fresh discover batch
Documented B-12 (cluster step chains unrelated articles into mega-clusters
via transitive connected-components grouping) in Master Doc §13 and
TRACKSHEET change log + M9 notes.

Processed evt_2026_06_28_040 (US strikes Iran after cargo ship attack,
16 articles spanning center-left/center/center-right). Total events: 15.

Ran scale_test.py --discover for fresh June 28 articles, adding ~1,500
new raw clusters to the candidate pool for future batches.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Milestones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Change Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="G14" s="32" t="inlineStr">
         <is>
-          <t>2026-06-01 — Scale test runner written (scripts/scale_test.py). B-01/B-02 enforced in reconcile.py. Awaiting G to run --discover and --run-events locally.</t>
+          <t>2026-06-01 — Scale test runner written (scripts/scale_test.py). B-01/B-02 enforced in reconcile.py. Awaiting G to run --discover and --run-events locally. | 2026-06-28 -- 4 more events processed (total 14/20-30). B-12 (clustering chaining into mega-clusters) flagged as backlog -- reduces usable candidate pool per discover run.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -2650,6 +2650,33 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Session 12/13 — 4 more events processed; B-12 clustering backlog flagged</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Committed/pushed session 11 work (Vercel deploy, B-10/B-11 fixes) plus a fix for generate.py crashing on bare-array model responses. Regenerated evt_014/062/066 with B-11 fix. Ran 4 new events: evt_2026_06_04_017 (UN Israel/Russia blacklist), evt_2026_06_01_023 (Iran-US ceasefire), evt_2026_06_01_117 (Beirut/Lebanon strikes), evt_2026_06_04_023 (Knesset dissolution bill). Total events now 14/20-30 target. Ran scale_test.py --discover for fresh June 28 articles; found only 1 clean diverse fresh cluster (evt_2026_06_28_040, US strikes Iran over cargo ship attack) -- most other large clusters were either re-clusters of already-processed stories or a mega-cluster chaining unrelated Gaza stories together. Logged as B-12 in Master Doc Section 13.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>M9 scale target is 20-30 events; clustering chaining issue reduces the effective pool of usable candidates per discover run, worth fixing before scaling batch size further</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>G + Claude Code</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Add Session 13 handover doc; tracksheet cleanup
Logged the missing regenerate/bare-array-fix change log entry and
corrected the M9 event count (14 -> 15) to reflect evt_2026_06_28_040.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1011,7 +1011,7 @@
       </c>
       <c r="G14" s="32" t="inlineStr">
         <is>
-          <t>2026-06-01 — Scale test runner written (scripts/scale_test.py). B-01/B-02 enforced in reconcile.py. Awaiting G to run --discover and --run-events locally. | 2026-06-28 -- 4 more events processed (total 14/20-30). B-12 (clustering chaining into mega-clusters) flagged as backlog -- reduces usable candidate pool per discover run.</t>
+          <t>2026-06-01 — Scale test runner written (scripts/scale_test.py). B-01/B-02 enforced in reconcile.py. Awaiting G to run --discover and --run-events locally. | 2026-06-28 -- 4 more events processed (total 15/20-30, after evt_2026_06_28_040). B-12 (clustering chaining into mega-clusters) flagged as backlog -- reduces usable candidate pool per discover run.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -2651,27 +2651,54 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="19" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="19" t="inlineStr">
         <is>
           <t>Session 12/13 — 4 more events processed; B-12 clustering backlog flagged</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>Committed/pushed session 11 work (Vercel deploy, B-10/B-11 fixes) plus a fix for generate.py crashing on bare-array model responses. Regenerated evt_014/062/066 with B-11 fix. Ran 4 new events: evt_2026_06_04_017 (UN Israel/Russia blacklist), evt_2026_06_01_023 (Iran-US ceasefire), evt_2026_06_01_117 (Beirut/Lebanon strikes), evt_2026_06_04_023 (Knesset dissolution bill). Total events now 14/20-30 target. Ran scale_test.py --discover for fresh June 28 articles; found only 1 clean diverse fresh cluster (evt_2026_06_28_040, US strikes Iran over cargo ship attack) -- most other large clusters were either re-clusters of already-processed stories or a mega-cluster chaining unrelated Gaza stories together. Logged as B-12 in Master Doc Section 13.</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="19" t="inlineStr">
         <is>
           <t>M9 scale target is 20-30 events; clustering chaining issue reduces the effective pool of usable candidates per discover run, worth fixing before scaling batch size further</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E63" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Regenerated evt_014/062/066 with B-11 fix; bare-array generate fix</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Committed session 11's uncommitted work (Vercel deploy, B-10/B-11 fixes, ~950 raw clusters) which had never been committed. Regenerated evt_2026_06_04_014/062/066 (the 3 events run before B-11 was finalized) -- evt_062 had 2 paragraphs correctly reclassified contested-&gt;framing by the enforcement guard. evt_066 generation crashed (AttributeError: 'list' object has no attribute 'get') because the model returned a bare JSON array instead of {"paragraphs": [...]}; fixed generate_report() in pipeline/generate/generate.py to normalize that shape. GitHub push also failed due to an expired/invalid stored credential; resolved by generating a new PAT.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>B-11 fix needed validation on real data before trusting it for new batches; an unhandled response shape was blocking the very next event in queue</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>G + Claude Code</t>
         </is>

</xml_diff>

<commit_message>
Autonomous pipeline (auto_run + launchd) and event images (schema v0.3)
- pipeline/images/: Wikimedia Commons image stage — permissive licenses only
  (CC0/CC BY/CC BY-SA/PD), Haiku query generation + disqualify-then-pick
  selection, full attribution stored at event.image
- web: homepage thumbnails + event-page hero with license-compliant credit line
- scripts/auto_run.py: unattended discover→qualify→publish cycle with hard
  gates (size, outlets, cross-spectrum, bodies, cohesion, novelty, one-attempt)
- pipeline/run_event.py: extracted shared stage-3–5 orchestration from scale_test
- config/launchd: 4-hour schedule plist
- backfill: images attached to existing events; also commits the July 1
  Cowork session's 3 events that were left uncommitted
- docs: master doc §15, session-14 handover, tracksheet updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1011,7 +1011,7 @@
       </c>
       <c r="G14" s="32" t="inlineStr">
         <is>
-          <t>2026-06-01 — Scale test runner written. B-01/B-02 enforced in reconcile.py. | 2026-06-28 — 5 more events processed by Claude Code session (evt_040 + 4 others). Total 15/20-30. B-12 (cluster chaining) flagged. | 2026-06-29 — 4 more events processed (evt_031 Smotrich/NY parade 17art, evt_035 UN blacklist 10art, evt_120 Iran deal 23art, evt_129 Kuwait strike 12art). Total 19/20-30. Regenerated evt_014/062/066 with B-11 fix. B-13 (duplicate clusters on homepage) and B-14 (token cost analysis) logged in Master Doc §13.</t>
+          <t>2026-06-01 — Scale test runner written. B-01/B-02 enforced in reconcile.py. | 2026-06-28 — 5 more events processed by Claude Code session (evt_040 + 4 others). Total 15/20-30. B-12 (cluster chaining) flagged. | 2026-06-29 — 4 more events processed (evt_031 Smotrich/NY parade 17art, evt_035 UN blacklist 10art, evt_120 Iran deal 23art, evt_129 Kuwait strike 12art). Total 19/20-30. Regenerated evt_014/062/066 with B-11 fix. B-13 (duplicate clusters on homepage) and B-14 (token cost analysis) logged in Master Doc §13. | 2026-07-01 — 3 more events processed (Cowork session): evt_2026_07_01_026 (US envoys arrive Doha amid disputed Iran meeting plans, 7art), evt_2026_07_01_118 (Smotrich announces 3 Gaza settlements, 4art), evt_2026_07_01_175 (Iran-US Strait of Hormuz shipping dispute, 4art). Discover run also surfaced evt_015 (Haaretz-heavy, low diversity) and evt_092 (all right-leaning outlets) -- skipped as weaker corroboration candidates. Total 24/20-30. | 2026-07-06 — Pipeline automated: auto_run.py runs every 4h via launchd with qualification gates (see Change Log). Event images added (schema v0.3). Total 24/20-30; automation will accumulate the rest.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -2813,29 +2813,110 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="19" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="19" t="inlineStr">
         <is>
           <t>B-16 prompt fix implemented; found conflict with B-02; B-17 logged</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>Implemented the B-16 'ACTOR DISPUTES' prompt block in RECONCILE_SYSTEM (pipeline/analyze/reconcile.py), per Cowork's spec. Validated on the 3 named test events (evt_2026_06_04_066, evt_2026_06_28_040, evt_2026_06_04_062): the reconcile model now correctly merges actor disputes (e.g. Iran vs US on Kuwait airport responsibility) into single claims with parallel framing -- but the fix is being neutralized downstream. Result: 0/0/1 contested claims produced vs 3-5/3-5/2-3 expected. Root cause: B-02 strips any source appearing in both supported_by and contested_by down to supported_by only; for actor-dispute claims it's normal for every outlet to responsibly report both sides in one article, so B-02 can empty out contested_by entirely, after which B-09 demotes the claim away from 'contested'. Confirmed via log trace: 8/8 observed B-09 firings across the 3 events were directly preceded by a B-02 strip emptying contested_by. Three resolution options scoped in Master Doc B-16 status update; not yet decided/implemented -- pending G's input. Separately, while reviewing example claims, identified B-17: all 13 beat-config outlets are Western/Israeli, so actor-dispute claims can never contain a source reporting Iran's (or other regional state's) position as fact, only Western paraphrase of it. Logged as a new backlog item with credibility tradeoffs to weigh (state-controlled outlets vs. independent press) before any source-list change.</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="19" t="inlineStr">
         <is>
           <t>B-16's prompt change alone doesn't fix the contested-claims problem because an older guard (B-02) actively undoes it; needed a full trace through the pipeline to find the real interaction. B-17 surfaced naturally while reviewing concrete examples with G and is worth tracking even though it's a separate, bigger decision.</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="19" t="inlineStr">
         <is>
           <t>G + Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="19" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B70" s="19" t="inlineStr">
+        <is>
+          <t>Scale test -- 3 new events processed</t>
+        </is>
+      </c>
+      <c r="C70" s="19" t="inlineStr">
+        <is>
+          <t>Ran scale_test.py --discover (5 clusters found); selected evt_2026_07_01_026 (US-Iran Doha talks/Strait of Hormuz, 7 outlets), evt_2026_07_01_118 (Smotrich Gaza settlements, 4 outlets), evt_2026_07_01_175 (Iran-US shipping dispute, 4 outlets) for full pipeline run based on outlet diversity/spectrum spread. Skipped evt_015 (Haaretz-heavy: 4/6 articles same outlet) and evt_092 (all right-leaning outlets, no left/center representation) as weaker corroboration candidates. All 3 selected events analyzed/annotated/generated successfully. Total processed events: 24/20-30.</t>
+        </is>
+      </c>
+      <c r="D70" s="19" t="inlineStr">
+        <is>
+          <t>M9 scale target is 20-30 events; diversity-based selection keeps corroboration signal meaningful across the political spectrum</t>
+        </is>
+      </c>
+      <c r="E70" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude (Cowork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="19" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B71" s="19" t="inlineStr">
+        <is>
+          <t>Automation — auto_run.py + launchd (M9 area)</t>
+        </is>
+      </c>
+      <c r="C71" s="19" t="inlineStr">
+        <is>
+          <t>Pipeline now runs autonomously every 4 hours. New scripts/auto_run.py: ingest -&gt; cluster -&gt; qualify -&gt; analyze/annotate/generate -&gt; image -&gt; git commit+push (Vercel auto-deploys). Qualification gates codify the manual selection criteria: 4-40 articles, &gt;=3 distinct outlets, cross-spectrum (&gt;=1 left-of-center AND &gt;=1 right-of-center), &gt;=3 usable bodies, cohesion &gt;=0.65, &lt;=40% URL overlap with published events, one-attempt fingerprinting (data/logs/autorun/state.json). Max 2 events/cycle; failed events cleaned up, never published; only selected clusters written to data/events/. run_pipeline_for_event extracted to pipeline/run_event.py (shared with scale_test.py). launchd job com.critiqal.newsroom.autorun (plist in config/launchd/, installed to ~/Library/LaunchAgents). Documented in Master Doc s15a.</t>
+        </is>
+      </c>
+      <c r="D71" s="19" t="inlineStr">
+        <is>
+          <t>Owner decision: move from manual per-session batches to unattended operation for go-live; gates + report validation replace pre-publish human review (supersedes s7 mitigation)</t>
+        </is>
+      </c>
+      <c r="E71" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Fable 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="19" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B72" s="19" t="inlineStr">
+        <is>
+          <t>Schema v0.3 — event images (pipeline/images/)</t>
+        </is>
+      </c>
+      <c r="C72" s="19" t="inlineStr">
+        <is>
+          <t>New image stage: Wikimedia Commons search with license filter (CC0/CC BY/CC BY-SA/public domain only; NC/ND rejected), Haiku query generation + disqualify-then-pick candidate selection. event.image object added to per-event JSON (schema 0.2 -&gt; 0.3, additive): url, caption, credit, license, license_url, source_page. Front end renders homepage thumbnails and event-page hero with full attribution line (license requirement). All 24 existing events backfilled (~2/3 got images; rest correctly imageless). Key prompt guardrail: photos featuring identifiable people not central to the event are disqualified. Documented in Master Doc s15b.</t>
+        </is>
+      </c>
+      <c r="D72" s="19" t="inlineStr">
+        <is>
+          <t>Homepage/event pages needed imagery without copyright exposure (s7); Commons-only with attribution is the defensible path</t>
+        </is>
+      </c>
+      <c r="E72" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Fable 5)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracksheet: ID-collision fix + Actions go-live
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3002,27 +3002,54 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="19" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="19" t="inlineStr">
         <is>
           <t>B-17 RESOLVED (state-aligned outlets) + developing-news novelty + UI refinements</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="19" t="inlineStr">
         <is>
           <t>G's decision: include state-aligned outlets with alignment made prominent. Added RT News (europe, Russian state-controlled), Global Times (asia, Chinese state-controlled), Asharq Al-Awsat + Saudi Gazette (middle east, Saudi state-aligned). New state_alignment field end-to-end (beat config -&gt; Article -&gt; sources[] -&gt; UI). Enforced as perspective-not-corroboration: excluded from auto_run cross-spectrum gate and B-01 agreed tier count; reconcile/generate prompts require inline attribution ('Russian state-controlled RT reported...'). UI: flag marker on chips, red badge on outlet cards, About-page explanation. Novelty gate redefined: &gt;=50% new URLs required (same-articles block), overlapping prior events recorded as event.related_events and shown as 'Earlier coverage' box — developing stories now publish as linked follow-ups instead of being rejected as duplicates. Beat display label changed to 'Middle East'; event image moved from top hero into the report body after the lede paragraph.</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="19" t="inlineStr">
         <is>
           <t>Counter-Western perspectives requested by G with explicit alignment labeling; developing stories needed room to publish without homepage duplication</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E76" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Fable 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Fix cross-beat event ID collision + go-live via GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>GitHub Actions now runs the autonomous pipeline every 6h (repo made public for unlimited minutes; ANTHROPIC_API_KEY secret set via API; ~1s fast auth-check + self-diagnosing failure issues added). Root-caused a major frontend bug: unique_event_id() only checked one beat's dir, so every beat minted evt_&lt;date&gt;_auto_001/002/... and the IDs collided across beats — getEvent(id) returned the first (alphabetical) beat match, rendering one event multiple times while shadowing same-ID events in other beats (the 'China x3' dupes AND the missing Europe/Israel events / 18-vs-22 count were both this). Fixed: IDs now namespaced evt_&lt;date&gt;_&lt;beat&gt;_&lt;NNN&gt;, globally unique; renamed all existing auto events; deleted 2 redundant Khamenei funeral events. Live site now shows 24 distinct events across all beats, no dupes.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Duplicates/mismatches/missing events reported on the live site; all traced to one ID-collision bug</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>G + Claude Code (Fable 5)</t>
         </is>

</xml_diff>

<commit_message>
tracksheet: log B-13 semantic dedup + homepage grouping; drop stale LibreOffice lock
- Change Log row for the 2026-07-07 semantic-dedup gate + story-grouping work.
- Remove accidentally-committed .~lock.TRACKSHEET.xlsx# (stale editor lock).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -105,6 +105,10 @@
       <charset val="1"/>
       <family val="0"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="13">
@@ -212,7 +216,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -327,6 +331,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1032,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3029,29 +3036,56 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="19" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="19" t="inlineStr">
         <is>
           <t>Fix cross-beat event ID collision + go-live via GitHub Actions</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="19" t="inlineStr">
         <is>
           <t>GitHub Actions now runs the autonomous pipeline every 6h (repo made public for unlimited minutes; ANTHROPIC_API_KEY secret set via API; ~1s fast auth-check + self-diagnosing failure issues added). Root-caused a major frontend bug: unique_event_id() only checked one beat's dir, so every beat minted evt_&lt;date&gt;_auto_001/002/... and the IDs collided across beats — getEvent(id) returned the first (alphabetical) beat match, rendering one event multiple times while shadowing same-ID events in other beats (the 'China x3' dupes AND the missing Europe/Israel events / 18-vs-22 count were both this). Fixed: IDs now namespaced evt_&lt;date&gt;_&lt;beat&gt;_&lt;NNN&gt;, globally unique; renamed all existing auto events; deleted 2 redundant Khamenei funeral events. Live site now shows 24 distinct events across all beats, no dupes.</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="19" t="inlineStr">
         <is>
           <t>Duplicates/mismatches/missing events reported on the live site; all traced to one ID-collision bug</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E77" s="19" t="inlineStr">
         <is>
           <t>G + Claude Code (Fable 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B78" s="39" t="inlineStr">
+        <is>
+          <t>B-13 addressed — semantic dedup gate + homepage story-grouping</t>
+        </is>
+      </c>
+      <c r="C78" s="39" t="inlineStr">
+        <is>
+          <t>auto_run.py evaluate_cluster now compares the candidate cluster embedding centroid against the title+summary embedding of events published in the last 5 days (all beats): cosine &gt;=0.93 rejects as a duplicate (no LLM tokens); &gt;=0.85 folds the match into related_events so it publishes as a grouped development, not a new card. Added embed_texts() to pipeline/cluster/embed.py. Homepage getEventGroups() (web/lib/data.ts) collapses related_events chains into one card with earlier coverage nested under a Developing story strip (web/app/page.tsx). semantic_sim/semantic_match logged per cluster for threshold recalibration.</t>
+        </is>
+      </c>
+      <c r="D78" s="39" t="inlineStr">
+        <is>
+          <t>URL-overlap novelty only blocked the same ARTICLES; the same STORY re-clustered from a different article set still published as N cards (three Khamenei funeral cards, 2026-07-06). Semantic layer closes that gap; homepage grouping shows a multi-day story once.</t>
+        </is>
+      </c>
+      <c r="E78" s="39" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Opus 4.8)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cron to 12h (pre-launch cost control); Session 16 handover + docs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3029,27 +3029,54 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="19" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="19" t="inlineStr">
         <is>
           <t>Fix cross-beat event ID collision + go-live via GitHub Actions</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="19" t="inlineStr">
         <is>
           <t>GitHub Actions now runs the autonomous pipeline every 6h (repo made public for unlimited minutes; ANTHROPIC_API_KEY secret set via API; ~1s fast auth-check + self-diagnosing failure issues added). Root-caused a major frontend bug: unique_event_id() only checked one beat's dir, so every beat minted evt_&lt;date&gt;_auto_001/002/... and the IDs collided across beats — getEvent(id) returned the first (alphabetical) beat match, rendering one event multiple times while shadowing same-ID events in other beats (the 'China x3' dupes AND the missing Europe/Israel events / 18-vs-22 count were both this). Fixed: IDs now namespaced evt_&lt;date&gt;_&lt;beat&gt;_&lt;NNN&gt;, globally unique; renamed all existing auto events; deleted 2 redundant Khamenei funeral events. Live site now shows 24 distinct events across all beats, no dupes.</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="19" t="inlineStr">
         <is>
           <t>Duplicates/mismatches/missing events reported on the live site; all traced to one ID-collision bug</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E77" s="19" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Fable 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Cron slowed to 12h; credit-balance diagnostics</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Anthropic account ran out of API credits on 7 July -&gt; autonomous cron began failing every cycle (billing, not code). CI fast-check + runner now distinguish 'BALANCE EXHAUSTED' (HTTP 400 credit balance) from 'invalid key' (HTTP 401), and a mid-cycle exhaustion aborts remaining beats. Cron slowed from every 6h to every 12h (00:23 &amp; 12:23 UTC) as pre-launch cost control (GitHub compute is free; this reduces Anthropic credit burn). Documented the two-separate-meters economics in Master Doc header + workflow header: running locally does NOT reduce API cost; only volume does.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Owner topping up credits; wants slower cadence pre-launch to control spend</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>G + Claude Code (Fable 5)</t>
         </is>

</xml_diff>

<commit_message>
tracksheet: log Session 17 frontend design pass; drop stale LibreOffice lock
- Change Log: design-pass entry (tagline, About tab, wider layout, raised cap; commit c1a0e60)
- Remove accidentally-committed .~lock.TRACKSHEET.xlsx# (stale, from a dead session)
- gitignore LibreOffice .~lock.*# so it can't be committed again

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -106,8 +106,12 @@
       <family val="0"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -177,8 +181,13 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F7F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -201,6 +210,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -212,7 +235,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -327,6 +350,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1032,7 +1058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3056,29 +3082,56 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="19" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="19" t="inlineStr">
         <is>
           <t>Cron slowed to 12h; credit-balance diagnostics</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="19" t="inlineStr">
         <is>
           <t>Anthropic account ran out of API credits on 7 July -&gt; autonomous cron began failing every cycle (billing, not code). CI fast-check + runner now distinguish 'BALANCE EXHAUSTED' (HTTP 400 credit balance) from 'invalid key' (HTTP 401), and a mid-cycle exhaustion aborts remaining beats. Cron slowed from every 6h to every 12h (00:23 &amp; 12:23 UTC) as pre-launch cost control (GitHub compute is free; this reduces Anthropic credit burn). Documented the two-separate-meters economics in Master Doc header + workflow header: running locally does NOT reduce API cost; only volume does.</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="19" t="inlineStr">
         <is>
           <t>Owner topping up credits; wants slower cadence pre-launch to control spend</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E78" s="19" t="inlineStr">
         <is>
           <t>G + Claude Code (Fable 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="36" customHeight="1" s="20">
+      <c r="A79" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B79" s="39" t="inlineStr">
+        <is>
+          <t>Frontend — design pass (Session 17)</t>
+        </is>
+      </c>
+      <c r="C79" s="39" t="inlineStr">
+        <is>
+          <t>Claude-design UI update, committed c1a0e60 &amp; pushed to main (live on Vercel). Homepage (web/app/page.tsx): tagline -&gt; "Think critically. Read Critiqal." (italic 18px semibold); beat nav centered via justify-content:space-between; new About tab after Asia (links /about); content max-width 760-&gt;960 with 48px horizontal padding; removed agreed/contested counts from feed meta rows (date + outlet count only). Event page (web/app/event/[id]/page.tsx): max-width 720-&gt;960, top padding 44-&gt;24px, header margin-bottom 32-&gt;20px. Report (web/components/ReportView.tsx): raised cap on the lede's first letter (scoped .report-lede::first-letter, Spectral serif 3.6em bold, baseline-aligned — raised, not floating drop cap). globals.css/layout.tsx unchanged (tokens unchanged). tsc clean.</t>
+        </is>
+      </c>
+      <c r="D79" s="39" t="inlineStr">
+        <is>
+          <t>G's Claude-design revisions to widen the reading column, sharpen the masthead slogan, add About to the nav, and give the report a print-style raised initial.</t>
+        </is>
+      </c>
+      <c r="E79" s="39" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Opus 4.8)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 design: STAGE_7_ENTITIES.md draft + M10-M12 milestones
Design-first per G's Phase 3 command — no implementation code. Entity Cards
stage doc drafted (entity store, resolution logic, confidence tiers,
Wikidata grounding, v0.5 additive schema, B-10 degradation, cost estimate).

Flags for G: task_4517860d (semantic dedup) complete but unmerged on
claude/ecstatic-dubinsky-bd166c and conflicting with the Session 17 design
pass -> M11 (threading) blocked pending merge decision; person-card review
gate clashes with Master Doc §15a autonomy -> proposed ship-dark
review_status; allegation tier excluded for persons in v1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -235,7 +235,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -352,6 +352,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -607,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="19" min="1" max="1"/>
@@ -1038,6 +1044,117 @@
       <c r="G14" s="32" t="inlineStr">
         <is>
           <t>2026-06-01 — Scale test runner written. B-01/B-02 enforced in reconcile.py. | 2026-06-28 — 5 more events processed by Claude Code session (evt_040 + 4 others). Total 15/20-30. B-12 (cluster chaining) flagged. | 2026-06-29 — 4 more events processed (evt_031 Smotrich/NY parade 17art, evt_035 UN blacklist 10art, evt_120 Iran deal 23art, evt_129 Kuwait strike 12art). Total 19/20-30. Regenerated evt_014/062/066 with B-11 fix. B-13 (duplicate clusters on homepage) and B-14 (token cost analysis) logged in Master Doc §13. | 2026-07-01 — 3 more events processed (Cowork session): evt_2026_07_01_026 (US envoys arrive Doha amid disputed Iran meeting plans, 7art), evt_2026_07_01_118 (Smotrich announces 3 Gaza settlements, 4art), evt_2026_07_01_175 (Iran-US Strait of Hormuz shipping dispute, 4art). Discover run also surfaced evt_015 (Haaretz-heavy, low diversity) and evt_092 (all right-leaning outlets) -- skipped as weaker corroboration candidates. Total 24/20-30. | 2026-07-06 — Pipeline automated: auto_run.py runs every 4h via launchd with qualification gates (see Change Log). Event images added (schema v0.3). Total 24/20-30; automation will accumulate the rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>Entity Cards</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D15" s="40" t="inlineStr">
+        <is>
+          <t>STAGE_7_ENTITIES.md</t>
+        </is>
+      </c>
+      <c r="E15" s="40" t="inlineStr">
+        <is>
+          <t>Persistent entity store (data/entities/) + extraction/resolution/grounding stage; clickable, tier-labeled entity cards in transparency mode; person-card publish gate decided; schema v0.5</t>
+        </is>
+      </c>
+      <c r="F15" s="40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G15" s="40" t="inlineStr">
+        <is>
+          <t>Design doc drafted 2026-07-08 (Session 17), PENDING G REVIEW. Decisions needed: person-card review gate (clashes with §15a autonomy), no-allegations-for-persons v1, cost sign-off (~$0.02-0.05/event cold, Haiku+Wikidata). No implementation until approved + credits resolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Story Threading</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>STAGE_8_THREADING.md (not yet written)</t>
+        </is>
+      </c>
+      <c r="E16" s="40" t="inlineStr">
+        <is>
+          <t>Persistent thread_id groups events of one ongoing story; chronological thread view + what-changed summaries; supersedes related_events</t>
+        </is>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G16" s="40" t="inlineStr">
+        <is>
+          <t>BLOCKED 2026-07-08: prerequisite task_4517860d (semantic dedup + homepage grouping) is complete but UNMERGED on branch claude/ecstatic-dubinsky-bd166c, and now conflicts with the Session 17 design pass (web/app/page.tsx). Merge + reconcile first; threading design must extend that mechanism. Sequencing decision with G.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>Accountability Tracking</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="inlineStr">
+        <is>
+          <t>STAGE_9_ACCOUNTABILITY.md (not yet written)</t>
+        </is>
+      </c>
+      <c r="E17" s="40" t="inlineStr">
+        <is>
+          <t>Per-outlet claim history across a thread; contradiction/correction/retraction flags rendered in the transparency layer, parallel tone</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G17" s="40" t="inlineStr">
+        <is>
+          <t>Depends on M11 (threading). Design after STAGE_8 is approved. 2026-07-08.</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3135,6 +3252,33 @@
         </is>
       </c>
     </row>
+    <row r="80" ht="36" customHeight="1" s="20">
+      <c r="A80" s="41" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B80" s="41" t="inlineStr">
+        <is>
+          <t>Phase 3 kickoff — design docs (Session 17)</t>
+        </is>
+      </c>
+      <c r="C80" s="41" t="inlineStr">
+        <is>
+          <t>G's Phase 3 command (entity cards / story threading / accountability tracking) reviewed against repo. STAGE_7_ENTITIES.md drafted (design only, no code): persistent entity store data/entities/ with append-only facts, confidence tiers mirroring claim classification, Wikidata/Wikipedia grounding (free, cited) with Anthropic web-search fallback, event schema v0.4-&gt;v0.5 additive entities[] block, B-10 graceful degradation, cost est ~$0.02-0.05/event cold. Milestones M10-M12 added. FINDINGS: (1) task_4517860d semantic dedup is DONE but UNMERGED on branch claude/ecstatic-dubinsky-bd166c and conflicts with Session 17 page.tsx design pass -&gt; M11 blocked pending merge decision; (2) person-card human review clashes with Master Doc §15a full autonomy -&gt; proposed review_status field, person cards ship dark until approved; (3) allegation tier excluded for persons in v1 (defamation exposure).</t>
+        </is>
+      </c>
+      <c r="D80" s="41" t="inlineStr">
+        <is>
+          <t>Phase 3 command working rules: design-first, flag legal/trust risk, check task_4517860d before threading, cost estimate before implementation</t>
+        </is>
+      </c>
+      <c r="E80" s="41" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Fable 5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
STAGE_7 Entity Cards APPROVED with G's modifications
G approved the design to build, with four changes now folded into the doc:
- Each card carries an openly-licensed entity image (Wikidata P18 -> Commons,
  reusing Stage-15b license discipline; attribution mandatory).
- `location` is a first-class entity type (strategic "why here?" significance,
  e.g. Bushehr, Strait of Hormuz).
- No human-review bottleneck: person cards auto-publish (§15a autonomy intact),
  safeguarded by machine enforcement — a person fact cannot publish without
  both a source link and a tier label.
- Allegations about people allowed only as attributed, linked meta-coverage
  ("Alleged by [outlet] ->"), never asserted in the system's own voice.

review_status kept as a dormant schema hook. TRACKSHEET M10 + change log
updated. Implementation gated on Anthropic credit top-up (paid Haiku calls
to test the extract/relevance steps).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1080,7 +1080,7 @@
       </c>
       <c r="G15" s="40" t="inlineStr">
         <is>
-          <t>Design doc drafted 2026-07-08 (Session 17), PENDING G REVIEW. Decisions needed: person-card review gate (clashes with §15a autonomy), no-allegations-for-persons v1, cost sign-off (~$0.02-0.05/event cold, Haiku+Wikidata). No implementation until approved + credits resolved.</t>
+          <t>APPROVED by G 2026-07-08 with modifications: (1) each card carries an openly-licensed entity image (Wikidata P18 -&gt; Commons, attribution mandatory); (2) location is a first-class type (strategic 'why here?' significance, e.g. Bushehr/Strait of Hormuz); (3) NO human-review bottleneck — person cards auto-publish, safeguarded by machine enforcement (a person fact can't publish without a source LINK + a tier LABEL); (4) allegations about people allowed ONLY as attributed meta-coverage ('Alleged by [outlet] -&gt;' + link). STAGE_7 doc updated. Implementation gated on Anthropic credits confirmation (paid Haiku calls to test).</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3306,6 +3306,33 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="36" customHeight="1" s="20">
+      <c r="A82" s="41" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B82" s="41" t="inlineStr">
+        <is>
+          <t>Entity Cards (M10) APPROVED with modifications</t>
+        </is>
+      </c>
+      <c r="C82" s="41" t="inlineStr">
+        <is>
+          <t>G approved STAGE_7 to build, adding: (1) an openly-licensed entity image per card (reuses Stage-15b image/license discipline via Wikidata P18); (2) location promoted to a first-class entity type answering 'why does this place matter' (Bushehr, Strait of Hormuz…); (3) no human-review gate — person cards auto-publish, with machine enforcement as the safeguard (a person fact is dropped unless it has both a source link and a section-5 tier label); (4) allegations about people permitted only as attributed, linked meta-coverage, never the system's own assertion. Doc revised accordingly (approval banner, location type, image field/step, reworked safety gate, updated cost/handoff). review_status kept in schema as a dormant hook if a human glance is wanted later. Build gated on credit top-up.</t>
+        </is>
+      </c>
+      <c r="D82" s="41" t="inlineStr">
+        <is>
+          <t>G's decisions on the four open Phase-3 questions; sourcing+labeling discipline deemed sufficient safeguard in place of a human bottleneck, keeping §15a autonomy intact</t>
+        </is>
+      </c>
+      <c r="E82" s="41" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Opus 4.8)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
STAGE_8 Story Threading design doc + M11 in progress
Design-first per G's Phase 3 command — no implementation code. Persistent
cross-beat threads on a new "Developing" tab; explicit IDF-weighted
entity+theme+embedding matching rule over a 30-day window (powered by the
M10 entities); extends related_events/getEventGroups rather than competing
with it. G's decision baked in: a thread requires >=2 events, so a single
new report never appears as "developing." Event schema 0.5->0.6 planned
(additive thread_id). Pending G review before build.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1115,12 +1115,12 @@
       </c>
       <c r="F16" s="40" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G16" s="40" t="inlineStr">
         <is>
-          <t>Unblocked 2026-07-08: prerequisite semantic-dedup + homepage story-grouping (task_4517860d, branch claude/ecstatic-dubinsky-bd166c, B-13) MERGED to main and verified live. Threading design (STAGE_8) can now proceed as an extension of related_events/getEventGroups. Not yet written.</t>
+          <t>Design doc STAGE_8_THREADING.md drafted 2026-07-08, PENDING G REVIEW. Persistent cross-beat threads on a new 'Developing' tab; matching = IDF-weighted entity overlap + theme + embedding over a 30-day window (entities from M10 power it); extends related_events/getEventGroups (not a parallel system). G's rule baked in: a thread needs &gt;=2 events, so a single new report never shows as 'developing'. Decisions pending: thresholds, tab label, neutral-title constraint, backfill window. No code until approved.</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3390,6 +3390,33 @@
         </is>
       </c>
     </row>
+    <row r="85" ht="36" customHeight="1" s="20">
+      <c r="A85" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B85" s="39" t="inlineStr">
+        <is>
+          <t>M11 Story Threading — design doc (STAGE_8)</t>
+        </is>
+      </c>
+      <c r="C85" s="39" t="inlineStr">
+        <is>
+          <t>Drafted STAGE_8_THREADING.md (design only, no code). Persistent 'thread' objects (data/threads/) group the events of one developing story into a named, ordered arc, surfaced on a new cross-beat 'Developing' tab (G's park insight: news is always developing; readers want to click 'US-Iran negotiations' and see the whole arc). Explicit matching rule: IDF-weighted major-entity overlap (M10 entities) + claim_group theme + title/summary embedding, over a 30-day rolling window; requires &gt;=1 shared SPECIFIC entity to avoid gluing events that merely share 'Israel'/'US' (the B-12 failure at thread level). Prefers under-merging; never auto-merges two established threads (logged for review). Distinct from the shipped semantic dedup (same ARTICLES, 5-day) — threading links DIFFERENT reports on the same STORY over weeks. Event schema 0.5-&gt;0.6 (additive event.thread_id); subsumes getEventGroups. G's decision baked in: a thread only exists at &gt;=2 events, so a lone new report is never shown as 'developing'. AI thread titles are neutral + human-overridable (flagged as a trust risk). Cost ~$0.005-0.01 per threaded event (matching is free; only chapter/title summaries cost). Substrate for M12 Accountability.</t>
+        </is>
+      </c>
+      <c r="D85" s="39" t="inlineStr">
+        <is>
+          <t>Phase 3 feature 2; sequenced after entities (which power the matching) and the dedup merge (which it extends)</t>
+        </is>
+      </c>
+      <c r="E85" s="39" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Opus 4.8)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
STAGE_9 Accountability Tracking design doc + M12 in progress
Design-first per Phase 3 command — no implementation code. Final feature:
tracks where an outlet's OWN reporting contradicts/corrects/retracts itself
across a thread, shown in parallel language with both receipts ("X said A
on day 1, not-A on day 3"), never editorializing. Built on M11 threads;
reuses claim_id/source_id; thread schema 0.1->0.2 (additive). Central guard:
only flags same-fact self-reversal, never normal story developments.
Flagged to G as the highest trust/defamation-risk feature — recommends a
human-review gate before flags display. Pending G review before build.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1152,12 +1152,12 @@
       </c>
       <c r="F17" s="40" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G17" s="40" t="inlineStr">
         <is>
-          <t>Depends on M11 (threading). Design after STAGE_8 is approved. 2026-07-08.</t>
+          <t>Design doc STAGE_9_ACCOUNTABILITY.md drafted 2026-07-08, PENDING G REVIEW. Tracks where an outlet's OWN reporting contradicts/corrects/retracts itself across a thread (reuses claim_id/source_id; thread schema 0.1-&gt;0.2 additive accountability[]). Core guard: only flags same-fact self-reversal, never normal story developments (the world changing != the outlet erring). Rendered as a parallel, motive-free 'How the reporting changed' section on the thread page. Decisions pending: human-review gate (recommend YES given defamation stakes), Sonnet for detection. No code until approved.</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3444,6 +3444,33 @@
         </is>
       </c>
     </row>
+    <row r="87" ht="36" customHeight="1" s="20">
+      <c r="A87" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B87" s="39" t="inlineStr">
+        <is>
+          <t>M12 Accountability Tracking — design doc (STAGE_9)</t>
+        </is>
+      </c>
+      <c r="C87" s="39" t="inlineStr">
+        <is>
+          <t>Drafted STAGE_9_ACCOUNTABILITY.md (design only, no code) — the final Phase 3 feature. Tracks, ACROSS A THREAD, where an outlet's OWN reporting contradicts/corrects/retracts its earlier account of the SAME fact, shown side-by-side in parallel language with both receipts and dates — 'X said A on day 1, not-A on day 3, judge for yourself', never 'X is biased'. Built on M11 threads; reuses claim_id/source_id (no parallel IDs); thread schema 0.1-&gt;0.2 (additive accountability[]). THE central hazard, called out explicitly: most changes over a developing story are the STORY developing, not the outlet erring (ceasefire held-&gt;collapsed is accurate reporting, not a contradiction) — detection must fire ONLY on same-fact self-reversal and fail safe (flag nothing on doubt). Detection = one Sonnet call per thread-update per returning outlet (~$0.02-0.04, only when a thread extends); machine validator drops any flag missing either receipt or not resolving to the same outlet; every flag audit-logged + suppressible. Rendered as a collapsed 'How the reporting changed' section on the thread page. FLAGGED TO G (highest trust/defamation stakes of the three features): recommend a human-review gate so flags render only once approved (option b), vs fully autonomous high-bar+audit (option a). Completes Phase 3 design once approved.</t>
+        </is>
+      </c>
+      <c r="D87" s="39" t="inlineStr">
+        <is>
+          <t>Phase 3 feature 3; depends on threading; command rule 6 requires flagging legal/trust risk before building, and publicly asserting a named outlet contradicted itself is the riskiest thing the product does</t>
+        </is>
+      </c>
+      <c r="E87" s="39" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Opus 4.8)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
docs: Session 17 handover + master doc refresh (Phase 3 complete)
- docs/HANDOVER_SESSION_17.md: full session (design pass, B-13 dedup merge,
  Phase 3 M10/M11/M12), live state, new CLIs, open items, conventions.
- 00_MASTER_DOCUMENT.md: header -> Phase 3 complete / schema v0.6 /
  handover 17; §9 milestones +M10-M12 (Done); §10 doc map +STAGE_8/9.
- TRACKSHEET: handover + doc-refresh change-log entry.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TRACKSHEET.xlsx
+++ b/TRACKSHEET.xlsx
@@ -1178,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="19" min="1" max="1"/>
@@ -3498,6 +3498,33 @@
         </is>
       </c>
     </row>
+    <row r="89" ht="36" customHeight="1" s="20">
+      <c r="A89" s="39" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B89" s="39" t="inlineStr">
+        <is>
+          <t>Session 17 handover + documentation refresh</t>
+        </is>
+      </c>
+      <c r="C89" s="39" t="inlineStr">
+        <is>
+          <t>Wrote docs/HANDOVER_SESSION_17.md covering the whole session: frontend design pass, the B-13 semantic-dedup branch merge (was complete-but-unmerged), and all of Phase 3 (M10 entities + M11 threading + M12 accountability). Refreshed 00_MASTER_DOCUMENT.md: header now says Phase 3 complete / schema v0.6 / handover 17; §9 milestone table gains M10-M12 (Done); §10 doc map gains STAGE_8/STAGE_9; §15c/d/e document the three features. STAGE_7/8/9 status lines marked IMPLEMENTED. Live counts: 30 events, 157 entity records, 3 threads, 0 accountability flags. Noted the standing accountability review queue and the stale root-level doc duplicates (docs/ is canonical) as open items.</t>
+        </is>
+      </c>
+      <c r="D89" s="39" t="inlineStr">
+        <is>
+          <t>Session handover + keep the single source of truth current, per project convention</t>
+        </is>
+      </c>
+      <c r="E89" s="39" t="inlineStr">
+        <is>
+          <t>G + Claude Code (Opus 4.8)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>